<commit_message>
Valuation: DCF v4 with the full dated pipeline (170,200 m2; 'Otros proyectos Chile' activated, Exhibits v7), bear/bull redefined with all tornado levers, figure data and static model values refreshed, bear/bull illustration from the team
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188QZHBkA8n5QL7BtmFakQg
</commit_message>
<xml_diff>
--- a/secciones/valuacion/modelos/Mallplaza_Figuras_Valuacion.xlsx
+++ b/secciones/valuacion/modelos/Mallplaza_Figuras_Valuacion.xlsx
@@ -651,7 +651,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="44" min="1" max="1"/>
     <col width="95" customWidth="1" style="44" min="2" max="2"/>
@@ -874,7 +874,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -937,7 +937,7 @@
         <v/>
       </c>
       <c r="C5" s="55" t="n">
-        <v>5051</v>
+        <v>5121.7</v>
       </c>
       <c r="D5" s="56">
         <f>0.8*C5+0.2*2951.38547083101</f>
@@ -956,7 +956,7 @@
         <v/>
       </c>
       <c r="C6" s="55" t="n">
-        <v>4290</v>
+        <v>4344.6</v>
       </c>
       <c r="D6" s="56">
         <f>0.8*C6+0.2*2951.38547083101</f>
@@ -975,7 +975,7 @@
         <v/>
       </c>
       <c r="C7" s="55" t="n">
-        <v>3703</v>
+        <v>3744.8</v>
       </c>
       <c r="D7" s="56">
         <f>0.8*C7+0.2*2951.38547083101</f>
@@ -994,7 +994,7 @@
         <v/>
       </c>
       <c r="C8" s="55" t="n">
-        <v>3237</v>
+        <v>3268.1</v>
       </c>
       <c r="D8" s="56">
         <f>0.8*C8+0.2*2951.38547083101</f>
@@ -1013,7 +1013,7 @@
         <v/>
       </c>
       <c r="C9" s="55" t="n">
-        <v>2857</v>
+        <v>2880.4</v>
       </c>
       <c r="D9" s="56">
         <f>0.8*C9+0.2*2951.38547083101</f>
@@ -1032,7 +1032,7 @@
         <v/>
       </c>
       <c r="C10" s="55" t="n">
-        <v>2543</v>
+        <v>2559</v>
       </c>
       <c r="D10" s="56">
         <f>0.8*C10+0.2*2951.38547083101</f>
@@ -1051,7 +1051,7 @@
         <v/>
       </c>
       <c r="C11" s="55" t="n">
-        <v>2278</v>
+        <v>2288.5</v>
       </c>
       <c r="D11" s="56">
         <f>0.8*C11+0.2*2951.38547083101</f>
@@ -1070,7 +1070,7 @@
         <v/>
       </c>
       <c r="C12" s="55" t="n">
-        <v>2052</v>
+        <v>2057.7</v>
       </c>
       <c r="D12" s="56">
         <f>0.8*C12+0.2*2951.38547083101</f>
@@ -1089,7 +1089,7 @@
         <v/>
       </c>
       <c r="C13" s="55" t="n">
-        <v>1857</v>
+        <v>1858.7</v>
       </c>
       <c r="D13" s="56">
         <f>0.8*C13+0.2*2951.38547083101</f>
@@ -1108,7 +1108,7 @@
         <v/>
       </c>
       <c r="C14" s="55" t="n">
-        <v>1687</v>
+        <v>1685.3</v>
       </c>
       <c r="D14" s="56">
         <f>0.8*C14+0.2*2951.38547083101</f>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
       <c r="C15" s="55" t="n">
-        <v>1538</v>
+        <v>1533</v>
       </c>
       <c r="D15" s="56">
         <f>0.8*C15+0.2*2951.38547083101</f>
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="B17" s="61" t="n">
-        <v>0.0756146197226035</v>
+        <v>0.07600147401979046</v>
       </c>
       <c r="C17" s="49" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B19" s="61" t="n">
-        <v>0.0741153260304354</v>
+        <v>0.07450820058336567</v>
       </c>
       <c r="C19" s="49" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
     <row r="22" ht="15" customHeight="1" s="45">
       <c r="A22" s="49" t="inlineStr">
         <is>
-          <t>Mensaje: para justificar CLP 3.555 el mercado debe descontar a ~7,6% nominal (~4,4% real), 285 pb bajo nuestra WACC (ver V2).</t>
+          <t>Mensaje: para justificar CLP 3.555 el mercado debe descontar a ~7.60% nominal (~4.5% real). 281 pb bajo nuestra WACC terminal.</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F35"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -1786,7 +1786,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="110" customWidth="1" style="44" min="1" max="1"/>
   </cols>
@@ -1826,7 +1826,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:H87"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="58" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -3277,11 +3277,11 @@
         </is>
       </c>
       <c r="B77" s="55" t="n">
-        <v>2311</v>
+        <v>2323</v>
       </c>
       <c r="C77" s="49" t="inlineStr">
         <is>
-          <t>Réplica del DCF v2 con WACC −107 pb en todos los períodos</t>
+          <t>Réplica del DCF v4 con WACC -107 pb en todos los períodos</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
     <row r="81" ht="15" customHeight="1" s="45">
       <c r="A81" s="49" t="inlineStr">
         <is>
-          <t>Es la elección más conservadora: con el bono en pesos el precio objetivo sube a ~CLP 2.439, todavía 31% bajo el precio de CLP 3.555. La recomendación no cambia.</t>
+          <t>Es la elección más conservadora: con el bono en pesos el precio objetivo sube a ~CLP 2.449. todavía 31% bajo el precio.</t>
         </is>
       </c>
     </row>
@@ -3375,7 +3375,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" style="44" min="1" max="1"/>
     <col width="62" customWidth="1" style="44" min="2" max="2"/>
@@ -3683,7 +3683,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="44" min="1" max="1"/>
     <col width="26" customWidth="1" style="44" min="2" max="2"/>
@@ -4090,7 +4090,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" style="44" min="1" max="1"/>
     <col width="42" customWidth="1" style="44" min="2" max="2"/>
@@ -4370,7 +4370,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -4431,13 +4431,13 @@
         </is>
       </c>
       <c r="B5" s="55" t="n">
-        <v>1686.94389181781</v>
+        <v>1685.26566288299</v>
       </c>
       <c r="C5" s="55" t="n">
-        <v>2051.79933329428</v>
+        <v>2057.71807392741</v>
       </c>
       <c r="D5" s="55" t="n">
-        <v>1856.81199718015</v>
+        <v>1858.653397229331</v>
       </c>
       <c r="E5" s="49" t="inlineStr">
         <is>
@@ -4452,13 +4452,13 @@
         </is>
       </c>
       <c r="B6" s="55" t="n">
-        <v>1379.44188269913</v>
+        <v>1390.82641661259</v>
       </c>
       <c r="C6" s="55" t="n">
-        <v>2328.90760780526</v>
+        <v>2329.25866009222</v>
       </c>
       <c r="D6" s="55" t="n">
-        <v>1856.81199718015</v>
+        <v>1858.653397229331</v>
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
@@ -4473,13 +4473,13 @@
         </is>
       </c>
       <c r="B7" s="55" t="n">
-        <v>1893.65312381858</v>
+        <v>1894.99070297252</v>
       </c>
       <c r="C7" s="55" t="n">
-        <v>1893.65312381858</v>
+        <v>1894.99070297252</v>
       </c>
       <c r="D7" s="55" t="n">
-        <v>1893.65312381858</v>
+        <v>1894.99070297252</v>
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
@@ -4609,7 +4609,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="B11" s="61" t="n">
-        <v>0.0756146197226035</v>
+        <v>0.07600147401979046</v>
       </c>
       <c r="C11" s="60">
         <f>(1+B11)/(1+$B$4)-1</f>
@@ -4862,7 +4862,7 @@
     <row r="20" ht="15" customHeight="1" s="45">
       <c r="A20" s="49" t="inlineStr">
         <is>
-          <t>Lectura: a CLP 3.555 la WACC real implícita (~4,4%) supera en solo ~80 pb al costo real de la deuda de la propia Mallplaza (3,6%).</t>
+          <t>Lectura: a CLP 3.555 la WACC real implícita (~4.5%) supera el bono UF a 10 años del BCCh (2.5% real) y queda bajo la WACC de la tasación (5.55% real).</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -4935,7 +4935,7 @@
         </is>
       </c>
       <c r="B4" s="61" t="n">
-        <v>0.0690189707474264</v>
+        <v>0.07266032090359451</v>
       </c>
       <c r="C4" s="49" t="inlineStr">
         <is>
@@ -5077,10 +5077,10 @@
         <v/>
       </c>
       <c r="D14" s="55" t="n">
-        <v>582787.013869718</v>
+        <v>592936.212324403</v>
       </c>
       <c r="E14" s="55" t="n">
-        <v>1917.83874034918</v>
+        <v>1911.50630339501</v>
       </c>
       <c r="F14" s="58">
         <f>E14/$E$15-1</f>
@@ -5100,10 +5100,10 @@
         <v/>
       </c>
       <c r="D15" s="55" t="n">
-        <v>528835.311960595</v>
+        <v>540637.80850638</v>
       </c>
       <c r="E15" s="55" t="n">
-        <v>1856.81199718015</v>
+        <v>1858.65339722932</v>
       </c>
       <c r="F15" s="58">
         <f>E15/$E$15-1</f>
@@ -5123,10 +5123,10 @@
         <v/>
       </c>
       <c r="D16" s="55" t="n">
-        <v>474339.436361579</v>
+        <v>487810.963500129</v>
       </c>
       <c r="E16" s="55" t="n">
-        <v>1784.87985066846</v>
+        <v>1796.13741969812</v>
       </c>
       <c r="F16" s="58">
         <f>E16/$E$15-1</f>
@@ -5146,10 +5146,10 @@
         <v/>
       </c>
       <c r="D17" s="55" t="n">
-        <v>419299.387072671</v>
+        <v>434455.67730565</v>
       </c>
       <c r="E17" s="55" t="n">
-        <v>1699.49188081559</v>
+        <v>1721.69849194288</v>
       </c>
       <c r="F17" s="58">
         <f>E17/$E$15-1</f>
@@ -5310,7 +5310,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -5569,10 +5569,10 @@
         <v/>
       </c>
       <c r="D15" s="55" t="n">
-        <v>1888.8</v>
+        <v>1892.2</v>
       </c>
       <c r="E15" s="56">
-        <f>0.8*D15+0.2*2951.38547083101</f>
+        <f>0.8*D15+0.19999999999999996*2951.38547083101</f>
         <v/>
       </c>
       <c r="F15" s="58">
@@ -5594,10 +5594,10 @@
         <v/>
       </c>
       <c r="D16" s="55" t="n">
-        <v>1872.8</v>
+        <v>1875.4</v>
       </c>
       <c r="E16" s="56">
-        <f>0.8*D16+0.2*2951.38547083101</f>
+        <f>0.8*D16+0.19999999999999996*2951.38547083101</f>
         <v/>
       </c>
       <c r="F16" s="58">
@@ -5619,10 +5619,10 @@
         <v/>
       </c>
       <c r="D17" s="55" t="n">
-        <v>1856.8</v>
+        <v>1858.7</v>
       </c>
       <c r="E17" s="56">
-        <f>0.8*D17+0.2*2951.38547083101</f>
+        <f>0.8*D17+0.19999999999999996*2951.38547083101</f>
         <v/>
       </c>
       <c r="F17" s="58">
@@ -5644,10 +5644,10 @@
         <v/>
       </c>
       <c r="D18" s="55" t="n">
-        <v>1840.8</v>
+        <v>1841.9</v>
       </c>
       <c r="E18" s="56">
-        <f>0.8*D18+0.2*2951.38547083101</f>
+        <f>0.8*D18+0.19999999999999996*2951.38547083101</f>
         <v/>
       </c>
       <c r="F18" s="58">
@@ -5669,10 +5669,10 @@
         <v/>
       </c>
       <c r="D19" s="55" t="n">
-        <v>1824.8</v>
+        <v>1825.2</v>
       </c>
       <c r="E19" s="56">
-        <f>0.8*D19+0.2*2951.38547083101</f>
+        <f>0.8*D19+0.19999999999999996*2951.38547083101</f>
         <v/>
       </c>
       <c r="F19" s="58">
@@ -5690,7 +5690,7 @@
     <row r="22" ht="15" customHeight="1" s="45">
       <c r="A22" s="49" t="inlineStr">
         <is>
-          <t>Lectura: todo el capital de trabajo vale ~CLP 32 por acción (1,7% del DCF). El valor no depende de este supuesto.</t>
+          <t>Lectura: todo el capital de trabajo vale ~CLP 33 por acción (1.8% del DCF). El valor no depende de este supuesto.</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5715,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="52" customWidth="1" style="44" min="1" max="1"/>
     <col width="15" customWidth="1" style="44" min="2" max="8"/>
@@ -5831,7 +5831,7 @@
         </is>
       </c>
       <c r="B9" s="59" t="n">
-        <v>0.100857870301779</v>
+        <v>0.100782648605333</v>
       </c>
       <c r="C9" s="58" t="n"/>
       <c r="D9" s="58" t="inlineStr">
@@ -5847,7 +5847,7 @@
         </is>
       </c>
       <c r="B10" s="59" t="n">
-        <v>0.112715304010366</v>
+        <v>0.112715864805192</v>
       </c>
       <c r="C10" s="58" t="n"/>
       <c r="D10" s="58" t="inlineStr">

</xml_diff>

<commit_message>
Informe final: Resumen de inversión con escenarios, sensibilidades y figuras R1–R3; Riesgos con cifras v4; Typst con tablas y figuras anchas; corrige referencias de anexos y cifras obsoletas (ESG, macro, V7); PDF ES/EN de 20 páginas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188QZHBkA8n5QL7BtmFakQg
</commit_message>
<xml_diff>
--- a/secciones/valuacion/modelos/Mallplaza_Figuras_Valuacion.xlsx
+++ b/secciones/valuacion/modelos/Mallplaza_Figuras_Valuacion.xlsx
@@ -1652,7 +1652,7 @@
         <v/>
       </c>
       <c r="D26" s="56">
-        <f>0.8*1856.81199718015+0.2*C26</f>
+        <f>0.8*1858.653397229331+0.19999999999999996*C26</f>
         <v/>
       </c>
       <c r="E26" s="58">
@@ -1673,7 +1673,7 @@
         <v/>
       </c>
       <c r="D27" s="56">
-        <f>0.8*1856.81199718015+0.2*C27</f>
+        <f>0.8*1858.653397229331+0.19999999999999996*C27</f>
         <v/>
       </c>
       <c r="E27" s="58">
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="D28" s="56">
-        <f>0.8*1856.81199718015+0.2*C28</f>
+        <f>0.8*1858.653397229331+0.19999999999999996*C28</f>
         <v/>
       </c>
       <c r="E28" s="58">
@@ -1715,7 +1715,7 @@
         <v/>
       </c>
       <c r="D29" s="56">
-        <f>0.8*1856.81199718015+0.2*C29</f>
+        <f>0.8*1858.653397229331+0.19999999999999996*C29</f>
         <v/>
       </c>
       <c r="E29" s="58">
@@ -1736,7 +1736,7 @@
         <v/>
       </c>
       <c r="D30" s="56">
-        <f>0.8*1856.81199718015+0.2*C30</f>
+        <f>0.8*1858.653397229331+0.19999999999999996*C30</f>
         <v/>
       </c>
       <c r="E30" s="58">

</xml_diff>